<commit_message>
Add FastAPI webapp and update review sources
Introduces a standalone BanglishCheck web app under `Technical Project/webapp` with a FastAPI backend, static frontend, Docker/Compose setup, and VPS deployment configs (Caddy/Nginx/systemd), plus a copied shared `banglishcheck.py` module for app use. Updates technical docs to distinguish the Gradio demo from the self-hosted web app path. Also expands the literature review by adding and verifying foundational XAI papers in `papers.md`, `review_plan.md`, and the reading matrix.
</commit_message>
<xml_diff>
--- a/Literature Review/reading_matrix.xlsx
+++ b/Literature Review/reading_matrix.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reading matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Reading matrix" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Reading matrix'!$A$1:$M$21</definedName>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1735,6 +1735,433 @@
       </c>
       <c r="M21" s="2" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>G. Foundational XAI theory</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Doshi-Velez and Kim</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Towards A Rigorous Science of Interpretable Machine Learning</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2017, arXiv:1702.08608</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>foundational (not in zip)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Position paper; proposes a taxonomy for evaluating interpretability (application-grounded, human-grounded, functionally-grounded)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Argues the field lacks agreed definitions/metrics for interpretability and proposes how to evaluate it rigorously</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Pre-LLM; taxonomy built for classical ML models, not generative text explanations</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Must read</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>G. Foundational XAI theory</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Miller</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Explanation in Artificial Intelligence: Insights from the Social Sciences</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2019, Artificial Intelligence 267:1-38</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>foundational (not in zip)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Literature synthesis from philosophy, psychology and cognitive science on how humans explain things to each other</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Good explanations are contrastive, selective and social, not just accurate; AI explanations should mirror how humans naturally explain</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>English-language social-science literature only; no empirical test on AI users</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Must read</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>G. Foundational XAI theory</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Ehsan and Riedl</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Human-centered Explainable AI: Towards a Reflective Sociotechnical Approach</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2020, arXiv:2002.01092</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>foundational (not in zip)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Conceptual framework paper introducing Human-centered XAI (HCXAI) as a sociotechnical, reflective design approach</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Explanations must be designed with the social context and the specific user in mind, not treated as a purely technical add-on</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Framework-level; no language-specific or low-resource discussion</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Must read</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>G. Foundational XAI theory</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Liao, Gruen and Miller</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Questioning the AI: Informing Design Practices for Explainable AI User Experiences</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2020, CHI '20, pp.1-15</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>foundational (not in zip)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Interviews with 20 UX/design practitioners; builds an XAI question bank of prototypical user questions about AI</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Surfaces a gap between algorithm-driven XAI techniques and the actual questions users want answered</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Practitioner sample is English-speaking; question bank not validated for non-English or code-mixed users</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Should read</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>G. Foundational XAI theory</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Jacovi and Goldberg</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Towards Faithfully Interpretable NLP Systems: How Should We Define and Evaluate Faithfulness?</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2020, ACL 2020, pp.4198-4205</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>foundational (not in zip)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Opinion/position paper proposing a graded, behavior-based definition of faithfulness for NLP interpretability methods</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Faithfulness should be evaluated as a measurable, graded property tied to model behavior, not treated as binary or assumed</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Defines faithfulness in the abstract; does not test across languages or scripts</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Must read</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>B. Reliance on LLM explanations</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Bansal et al.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Does the Whole Exceed its Parts? The Effect of AI Explanations on Complementary Team Performance</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2021, CHI '21</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>foundational (not in zip)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Controlled human-subject experiments measuring team performance and reliance with vs. without AI explanations</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Explanations increased acceptance of AI recommendations regardless of correctness; did not reliably improve complementary team performance</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>English-speaking participants; tasks are general decision-making, not language or code-mixed tasks</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Must read</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>B. Reliance on LLM explanations</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Vasconcelos et al.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Explanations Can Reduce Overreliance on AI Systems During Decision-Making</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2023, PACM HCI 7(CSCW1), Article 129</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>foundational (not in zip)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Five online experiments (N=731) varying explanation type and the cost/difficulty of verifying them</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>People strategically decide whether to engage with an explanation; explanations reduce overreliance mainly when they lower the cost of verification</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>English-speaking crowdworkers; verification-cost framing not tested for low-resource or code-mixed text</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Must read</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M21"/>
   <dataValidations count="1">

</xml_diff>